<commit_message>
feat: Implementar función para redondear marcas de tiempo a la media hora más cercana
</commit_message>
<xml_diff>
--- a/data/Historico.xlsx
+++ b/data/Historico.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>NO_CONFIRMADO</t>
+          <t>ELIMINADO</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NO_CONFIRMADO</t>
+          <t>ELIMINADO</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>NO_CONFIRMADO</t>
+          <t>ELIMINADO</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>NO_CONFIRMADO</t>
+          <t>ELIMINADO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1365,6 +1365,178 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>fcb5e822-760e-433e-ba7c-959657135f84</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ELIMINADO</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MILAGROS</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>46111.33333333334</v>
+      </c>
+      <c r="E23" s="1" t="n">
+        <v>46111.83333333334</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H23" t="n">
+        <v>70000</v>
+      </c>
+      <c r="I23" t="n">
+        <v>12</v>
+      </c>
+      <c r="J23" t="n">
+        <v>8</v>
+      </c>
+      <c r="K23" t="n">
+        <v>4</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>6da7e4d7-354b-4480-b8e8-fe0d27c59b22</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ELIMINADO</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>VANESA</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>46112.33333333334</v>
+      </c>
+      <c r="E24" s="1" t="n">
+        <v>46112.70833333334</v>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="n">
+        <v>9500</v>
+      </c>
+      <c r="H24" t="n">
+        <v>95000</v>
+      </c>
+      <c r="I24" t="n">
+        <v>9</v>
+      </c>
+      <c r="J24" t="n">
+        <v>7</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>70482157-87f3-4e22-b8cb-725d01d3dd0b</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ELIMINADO</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MILAGROS</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>46114.33333333334</v>
+      </c>
+      <c r="E25" s="1" t="n">
+        <v>46114.97916666666</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H25" t="n">
+        <v>102500</v>
+      </c>
+      <c r="I25" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="J25" t="n">
+        <v>8</v>
+      </c>
+      <c r="K25" t="n">
+        <v>5</v>
+      </c>
+      <c r="L25" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2b7625ff-4012-4124-98e8-62b3050c2c92</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>NO_CONFIRMADO</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>DANTE HERRERA</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>46118.33333333334</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>46118.70833333334</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>12000</v>
+      </c>
+      <c r="H26" t="n">
+        <v>108000</v>
+      </c>
+      <c r="I26" t="n">
+        <v>9</v>
+      </c>
+      <c r="J26" t="n">
+        <v>9</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>